<commit_message>
v6 Fig.7: dots only at round starts and candidate removals; 'judgment' renamed 'test' with a one-line definition
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig7_v6_mixT.xlsx
+++ b/figs/data/fig7_v6_mixT.xlsx
@@ -178,16 +178,9 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="circle"/>
-            <size val="4"/>
+            <symbol val="none"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2A78D6"/>
-              </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:solidFill>
-                  <a:srgbClr val="2A78D6"/>
-                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -207,6 +200,46 @@
         <ser>
           <idx val="1"/>
           <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'그림7 v6 학습'!AH1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림7 v6 학습'!$C$2:$C$29</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림7 v6 학습'!$AH$2:$AH$29</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!E1</f>
@@ -241,8 +274,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!G1</f>
@@ -277,8 +310,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="3"/>
-          <order val="3"/>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!I1</f>
@@ -313,8 +346,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="4"/>
-          <order val="4"/>
+          <idx val="5"/>
+          <order val="5"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!K1</f>
@@ -349,8 +382,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="5"/>
-          <order val="5"/>
+          <idx val="6"/>
+          <order val="6"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!M1</f>
@@ -385,8 +418,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="6"/>
-          <order val="6"/>
+          <idx val="7"/>
+          <order val="7"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!O1</f>
@@ -421,8 +454,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="7"/>
-          <order val="7"/>
+          <idx val="8"/>
+          <order val="8"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!Q1</f>
@@ -460,8 +493,8 @@
           </yVal>
         </ser>
         <ser>
-          <idx val="8"/>
-          <order val="8"/>
+          <idx val="9"/>
+          <order val="9"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!S1</f>
@@ -499,8 +532,8 @@
           </yVal>
         </ser>
         <ser>
-          <idx val="9"/>
-          <order val="9"/>
+          <idx val="10"/>
+          <order val="10"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!U1</f>
@@ -538,8 +571,8 @@
           </yVal>
         </ser>
         <ser>
-          <idx val="10"/>
-          <order val="10"/>
+          <idx val="11"/>
+          <order val="11"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!W1</f>
@@ -577,8 +610,8 @@
           </yVal>
         </ser>
         <ser>
-          <idx val="11"/>
-          <order val="11"/>
+          <idx val="12"/>
+          <order val="12"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!Y1</f>
@@ -616,8 +649,8 @@
           </yVal>
         </ser>
         <ser>
-          <idx val="12"/>
-          <order val="12"/>
+          <idx val="13"/>
+          <order val="13"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!AA1</f>
@@ -655,8 +688,8 @@
           </yVal>
         </ser>
         <ser>
-          <idx val="13"/>
-          <order val="13"/>
+          <idx val="14"/>
+          <order val="14"/>
           <tx>
             <strRef>
               <f>'그림7 v6 학습'!AC1</f>
@@ -758,10 +791,6 @@
     <legend>
       <legendPos val="b"/>
       <legendEntry>
-        <idx val="1"/>
-        <delete val="1"/>
-      </legendEntry>
-      <legendEntry>
         <idx val="2"/>
         <delete val="1"/>
       </legendEntry>
@@ -807,6 +836,10 @@
       </legendEntry>
       <legendEntry>
         <idx val="13"/>
+        <delete val="1"/>
+      </legendEntry>
+      <legendEntry>
+        <idx val="14"/>
         <delete val="1"/>
       </legendEntry>
     </legend>
@@ -1132,7 +1165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE528"/>
+  <dimension ref="A1:AH528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1150,6 +1183,11 @@
           <t>남은 후보 수 (파티션 2)</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>점: 회차 시작·후보 버린 순간 x</t>
+        </is>
+      </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>초기화1 x</t>
@@ -1217,7 +1255,7 @@
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>1회차 / YCSB-A+OLTP / 0.0~2.2h · 판단 267번</t>
+          <t>1회차 / YCSB-A+OLTP / 0.0~2.2h · 시험 267번</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
@@ -1227,7 +1265,7 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>2회차 / Varmail / 2.2~3.5h · 판단 1076번</t>
+          <t>2회차 / Varmail / 2.2~3.5h · 시험 1076번</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
@@ -1237,7 +1275,7 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>3회차 / YCSB-A+YCSB-B / 3.5~5.6h · 판단 47번</t>
+          <t>3회차 / YCSB-A+YCSB-B / 3.5~5.6h · 시험 47번</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
@@ -1247,7 +1285,7 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>4회차 / FIO-Fast / 5.6~6.7h · 판단 312번</t>
+          <t>4회차 / FIO-Fast / 5.6~6.7h · 시험 312번</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
@@ -1257,7 +1295,7 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>5회차 / Varmail / 6.7~7.9h · 판단 1034번</t>
+          <t>5회차 / Varmail / 6.7~7.9h · 시험 1034번</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
@@ -1267,7 +1305,7 @@
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>6회차 / YCSB-A / 8.0~9.0h · 판단 47번</t>
+          <t>6회차 / YCSB-A / 8.0~9.0h · 시험 47번</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
@@ -1277,7 +1315,12 @@
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>7회차 / OLTP / 9.0~10.0h · 판단 230번</t>
+          <t>7회차 / OLTP / 9.0~10.0h · 시험 230번</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>회차 시작·후보 버린 순간</t>
         </is>
       </c>
     </row>
@@ -1288,6 +1331,9 @@
       <c r="B2" t="n">
         <v>45</v>
       </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
@@ -1365,6 +1411,9 @@
       </c>
       <c r="AC2" t="n">
         <v>1</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -1374,6 +1423,9 @@
       <c r="B3" t="n">
         <v>45</v>
       </c>
+      <c r="C3" t="n">
+        <v>0.1648</v>
+      </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
@@ -1409,6 +1461,9 @@
       </c>
       <c r="O3" t="n">
         <v>48</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -1418,6 +1473,12 @@
       <c r="B4" t="n">
         <v>45</v>
       </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1426,6 +1487,12 @@
       <c r="B5" t="n">
         <v>45</v>
       </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1434,6 +1501,12 @@
       <c r="B6" t="n">
         <v>45</v>
       </c>
+      <c r="C6" t="n">
+        <v>2.9362</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1442,6 +1515,12 @@
       <c r="B7" t="n">
         <v>45</v>
       </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1450,6 +1529,12 @@
       <c r="B8" t="n">
         <v>45</v>
       </c>
+      <c r="C8" t="n">
+        <v>3.141</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1458,6 +1543,12 @@
       <c r="B9" t="n">
         <v>45</v>
       </c>
+      <c r="C9" t="n">
+        <v>3.1442</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1466,6 +1557,12 @@
       <c r="B10" t="n">
         <v>45</v>
       </c>
+      <c r="C10" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1474,6 +1571,12 @@
       <c r="B11" t="n">
         <v>45</v>
       </c>
+      <c r="C11" t="n">
+        <v>4.0426</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1482,6 +1585,12 @@
       <c r="B12" t="n">
         <v>45</v>
       </c>
+      <c r="C12" t="n">
+        <v>4.0435</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1490,6 +1599,12 @@
       <c r="B13" t="n">
         <v>45</v>
       </c>
+      <c r="C13" t="n">
+        <v>4.0551</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1498,6 +1613,12 @@
       <c r="B14" t="n">
         <v>45</v>
       </c>
+      <c r="C14" t="n">
+        <v>4.0648</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1506,6 +1627,12 @@
       <c r="B15" t="n">
         <v>45</v>
       </c>
+      <c r="C15" t="n">
+        <v>4.0909</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1514,6 +1641,12 @@
       <c r="B16" t="n">
         <v>45</v>
       </c>
+      <c r="C16" t="n">
+        <v>4.1402</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1522,6 +1655,12 @@
       <c r="B17" t="n">
         <v>45</v>
       </c>
+      <c r="C17" t="n">
+        <v>4.1499</v>
+      </c>
+      <c r="AH17" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1530,6 +1669,12 @@
       <c r="B18" t="n">
         <v>43</v>
       </c>
+      <c r="C18" t="n">
+        <v>4.1576</v>
+      </c>
+      <c r="AH18" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1538,6 +1683,12 @@
       <c r="B19" t="n">
         <v>43</v>
       </c>
+      <c r="C19" t="n">
+        <v>4.1605</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1546,6 +1697,12 @@
       <c r="B20" t="n">
         <v>43</v>
       </c>
+      <c r="C20" t="n">
+        <v>4.1683</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1554,6 +1711,12 @@
       <c r="B21" t="n">
         <v>43</v>
       </c>
+      <c r="C21" t="n">
+        <v>4.1896</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1562,6 +1725,12 @@
       <c r="B22" t="n">
         <v>43</v>
       </c>
+      <c r="C22" t="n">
+        <v>4.1925</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1570,6 +1739,12 @@
       <c r="B23" t="n">
         <v>43</v>
       </c>
+      <c r="C23" t="n">
+        <v>4.1934</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1578,6 +1753,12 @@
       <c r="B24" t="n">
         <v>43</v>
       </c>
+      <c r="C24" t="n">
+        <v>4.2108</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1586,6 +1767,12 @@
       <c r="B25" t="n">
         <v>43</v>
       </c>
+      <c r="C25" t="n">
+        <v>4.2118</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1594,6 +1781,12 @@
       <c r="B26" t="n">
         <v>43</v>
       </c>
+      <c r="C26" t="n">
+        <v>4.2253</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1602,6 +1795,12 @@
       <c r="B27" t="n">
         <v>43</v>
       </c>
+      <c r="C27" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1610,6 +1809,12 @@
       <c r="B28" t="n">
         <v>43</v>
       </c>
+      <c r="C28" t="n">
+        <v>5.9362</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1617,6 +1822,12 @@
       </c>
       <c r="B29" t="n">
         <v>43</v>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="30">

</xml_diff>